<commit_message>
analysis(AVGO): refresh post-Q2 FY26 print (June 3, 2026)
Q2 FY26 dropped today: revenue $22.2B (+48%, AI $10.8B +143%, adj EBITDA $15.2B/69%,
FCF $10.3B). Q3 guide $29.4B (+84% YoY). Stock +4.7% on the print to ~$481.62.

Key narrative refinement: Hock Tan REITERATED but did NOT raise the FY27 "AI $100B+"
guide despite the Q2 beat. Base-case haircut reduced from 24% to 15% (FY27 AI now
$85B, was $76B). Updated model, comps, deck, HTML with post-Q2 figures.

Refreshed outputs:
- DCF base implied/share: $246 -> $264 (sensitivity grid $200-311; was $185-289)
- Current price: $460 -> $482; gap: -47% -> -45%
- TTM revenue: $68.3B -> $75.5B; TTM FCF: $28.9B -> $33B+; net debt: $52B -> $49B
- Structural finding holds: market still embeds the bull AI ramp; even the
  most generous WACC/g corner ($395) is below the post-print price.

https://claude.ai/code/session_01VCX3Tmx1dtT8qoz4oxMuri
</commit_message>
<xml_diff>
--- a/analysis/AVGO/AVGO-Comps-Analysis.xlsx
+++ b/analysis/AVGO/AVGO-Comps-Analysis.xlsx
@@ -237,42 +237,42 @@
   <commentList>
     <comment ref="C7" authorId="0" shapeId="0">
       <text>
-        <t>AVGO ~$460/sh x ~4.73B sh, June 1 2026 (~$2.18T)</t>
+        <t>AVGO ~$481.62/sh post-Q2 FY26 (+4.7% on print) x ~4.73B sh = ~$2.28T (June 3, 2026)</t>
       </text>
     </comment>
     <comment ref="D7" authorId="0" shapeId="0">
       <text>
-        <t>Net debt = $66.06B debt - $14.2B cash (Q1 FY26 8-K, Feb 1 2026)</t>
+        <t>[E] Net debt ~$49B at May 3, 2026 (debt ~$65B - cash ~$16B; Q2 FCF $10.3B added)</t>
       </text>
     </comment>
     <comment ref="E7" authorId="0" shapeId="0">
       <text>
-        <t>[E] TTM revenue ~$68.3B (FY25 $63.9B + Q1 FY26 step-up)</t>
+        <t>TTM revenue $75.47B: Q3-Q4 FY25 ($15.95B+$18.02B) + Q1-Q2 FY26 ($19.3B+$22.2B)</t>
       </text>
     </comment>
     <comment ref="F7" authorId="0" shapeId="0">
       <text>
-        <t>Q1 FY26 revenue +29% YoY (Broadcom IR, Mar 2026)</t>
+        <t>Q2 FY26 revenue +48% YoY (Broadcom Q2 FY26 IR, June 3 2026); Q3 guide +84%</t>
       </text>
     </comment>
     <comment ref="G7" authorId="0" shapeId="0">
       <text>
-        <t>[E] GAAP gross margin ~68% (non-GAAP ~77%); Q1 FY26</t>
+        <t>[E] GAAP gross margin ~68% (non-GAAP ~77%); Q2 FY26</t>
       </text>
     </comment>
     <comment ref="H7" authorId="0" shapeId="0">
       <text>
-        <t>[E] TTM GAAP EBITDA ~$40.5B (NI + interest + tax + D&amp;A; adj. EBITDA ~$46B)</t>
+        <t>[E] TTM GAAP EBITDA ~$50.5B (adj EBITDA TTM ~$54B; Q2 adj EBITDA $15.2B / 69% margin)</t>
       </text>
     </comment>
     <comment ref="I7" authorId="0" shapeId="0">
       <text>
-        <t>[E] TTM GAAP net income ~$25.0B</t>
+        <t>[E] TTM GAAP net income ~$28.0B (Q2 GAAP NI $9.3B; non-GAAP $12.1B)</t>
       </text>
     </comment>
     <comment ref="J7" authorId="0" shapeId="0">
       <text>
-        <t>Forward P/E ~31x (StockAnalysis, consensus FY26-27)</t>
+        <t>[E] Forward P/E ~29x post-Q2 (consensus FY26-27 EPS upward revision absorbing the +48%)</t>
       </text>
     </comment>
     <comment ref="C8" authorId="0" shapeId="0">
@@ -841,7 +841,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>As of ~June 1, 2026 | $ in millions except ratios | Stats computed over the 5 semis peers (NVDA, AMD, MRVL, QCOM, TXN); AVGO = target, ORCL = software anchor (memo)</t>
+          <t>As of June 3, 2026 (post-AVGO Q2 FY26 print) | $ in millions except ratios | Stats over 5 semis peers (NVDA, AMD, MRVL, QCOM, TXN); AVGO=target, ORCL=software anchor (memo)</t>
         </is>
       </c>
     </row>
@@ -921,28 +921,28 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>2175800</v>
+        <v>2278000</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>51857</v>
+        <v>49000</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>68300</v>
+        <v>75470</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>0.29</v>
+        <v>0.48</v>
       </c>
       <c r="G7" s="8" t="n">
         <v>0.68</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>40500</v>
+        <v>50500</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>25000</v>
+        <v>28000</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K7" s="10" t="inlineStr">
         <is>

</xml_diff>